<commit_message>
second update 21_7 reading
</commit_message>
<xml_diff>
--- a/READING/1_21_07.xlsx
+++ b/READING/1_21_07.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\READING\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4EDD6B-C192-41F3-ABE7-F9BAC51552BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FD0021-8961-43FE-A10C-7577D067919D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16320" yWindow="885" windowWidth="27840" windowHeight="20040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="282">
   <si>
     <t>Fre</t>
   </si>
@@ -400,13 +400,679 @@
   </si>
   <si>
     <t>积累；装载；堆积</t>
+  </si>
+  <si>
+    <t>...てから</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>在…之后</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>片付く</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>かたづく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>整理好；收拾整齐；解决；处理好</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ております</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)处于…状态(2)正在…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>同"ている"</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>間に合う</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>赶得上；来得及</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>進める</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>すすめる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>推进；促进；进行</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>私の場合</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于我来说…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>おそらく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>恐怕</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>みたいに</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>～たとたん（に）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>刚一…就…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>像…一样</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>急に</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>突然；忽然</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>頭が固い</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>あたまがかたい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>思想顽固</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ような</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>像…那样</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>普通</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふつう</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>常见，平常</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>けれども</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>但是</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ないといけない</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>没有…是不行的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>要するに</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ようするに</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>总之；简而言之</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>アドバイス</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>advice</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>次第で</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>根据…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>意欲</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>干劲</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>授業</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>课堂，教学</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>かける</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动向对方发起的动作</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>好きに</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>自由地；尽情地</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>異なる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>不同;不一样</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>決まり</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>规定；规矩；决定</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>何か</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>某事；某物</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>つくる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>制作；创造</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>つける</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"-&gt;附着;添加"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>かける</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"-&gt;花费</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>見つけ出す</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(主动)发掘</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>仕方</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>方法；办法；做法</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ではないか</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)难道不是…吗(2)是否…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>すれ違い</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>擦肩而过</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>近づく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ちかづく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>靠近；接近</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>すれちがい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>甘やかされる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>被溺爱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>遭遇</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>そうぐう</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>遇到</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>"である"-&gt;"です"</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>シグナル</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>信号；标志</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>なんなのか</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>到底是什么</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>あるなし</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>にしたがった</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>遵从，遵守</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>たほうがよい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>最好…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>または</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>或者</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>“あるいは”-&gt;或者；有时</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>にもとづいて</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>基于；以...为基础</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>けが</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>受伤；负伤</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>身につける</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>学会；掌握</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>いやいや</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>不情愿的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>本格的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>正式的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>私達</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>我们</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>わたしたち</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>とんでもない</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)非常地…(2)惊人地(3)岂有此理；哪里的话</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>もったいない</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>浪费</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ぐらい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)到了…地步(程度)(2)大约</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>どんどん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>逐渐；越来越</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>退屈</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>たいくつ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>无聊；厌倦</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>そんなに</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>那样地</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>途方もない</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>无法想象;极其困难</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ますます</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>越来越</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>否応なく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>强制地。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>割り込む</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>わりこむ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>插入；打断；插队；插话</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>じゅうぶん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>足够；充分</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>耐えられる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>能够忍受</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>だけの</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>足以…的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ぜんぶ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>全部</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>切る</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)完全(2)切断</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>すくなく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>至少</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>あわただしい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>匆忙的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>済ませる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>完成</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>果たす</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>完成；实现；履行</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>はがき</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>明信片</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>問い合わせ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>咨询；询问</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>明記</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>明确记载；清楚写明</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>どちらか</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>哪一个；哪一方；哪个</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>開催日</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>かいさいび</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>举行日; 举办日</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>いたします</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>"します"谦让语</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,6 +1092,29 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="2">
@@ -463,11 +1152,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -770,13 +1464,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="26.375" customWidth="1"/>
     <col min="3" max="3" width="19.5" customWidth="1"/>
     <col min="4" max="4" width="29.125" customWidth="1"/>
+    <col min="5" max="5" width="45.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
@@ -1439,7 +2134,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A49">
         <v>0</v>
       </c>
@@ -1453,7 +2148,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A50">
         <v>0</v>
       </c>
@@ -1465,6 +2160,824 @@
       </c>
       <c r="D50" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A51">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>126</v>
+      </c>
+      <c r="D51" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A52">
+        <v>2</v>
+      </c>
+      <c r="B52" t="s">
+        <v>128</v>
+      </c>
+      <c r="C52" t="s">
+        <v>129</v>
+      </c>
+      <c r="D52" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A53">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>131</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D53" t="s">
+        <v>132</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A54">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>134</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A55">
+        <v>2</v>
+      </c>
+      <c r="B55" t="s">
+        <v>136</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D55" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A56">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>139</v>
+      </c>
+      <c r="D56" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A57">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>141</v>
+      </c>
+      <c r="D57" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A58">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>143</v>
+      </c>
+      <c r="D58" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A59">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>144</v>
+      </c>
+      <c r="D59" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A60">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>147</v>
+      </c>
+      <c r="D60" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A61">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>149</v>
+      </c>
+      <c r="C61" t="s">
+        <v>150</v>
+      </c>
+      <c r="D61" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A62">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>152</v>
+      </c>
+      <c r="D62" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A63">
+        <v>2</v>
+      </c>
+      <c r="B63" t="s">
+        <v>154</v>
+      </c>
+      <c r="C63" t="s">
+        <v>155</v>
+      </c>
+      <c r="D63" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A64">
+        <v>2</v>
+      </c>
+      <c r="B64" t="s">
+        <v>157</v>
+      </c>
+      <c r="D64" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A65">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>159</v>
+      </c>
+      <c r="D65" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A66">
+        <v>2</v>
+      </c>
+      <c r="B66" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" t="s">
+        <v>162</v>
+      </c>
+      <c r="D66" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A67">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>164</v>
+      </c>
+      <c r="D67" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A68">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>166</v>
+      </c>
+      <c r="D68" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A69">
+        <v>2</v>
+      </c>
+      <c r="B69" t="s">
+        <v>168</v>
+      </c>
+      <c r="D69" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A70">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>170</v>
+      </c>
+      <c r="D70" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A71">
+        <v>2</v>
+      </c>
+      <c r="B71" t="s">
+        <v>172</v>
+      </c>
+      <c r="D71" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A72">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>174</v>
+      </c>
+      <c r="D72" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A73">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>176</v>
+      </c>
+      <c r="D73" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A74">
+        <v>2</v>
+      </c>
+      <c r="B74" t="s">
+        <v>178</v>
+      </c>
+      <c r="D74" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A75">
+        <v>2</v>
+      </c>
+      <c r="B75" t="s">
+        <v>180</v>
+      </c>
+      <c r="D75" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A76">
+        <v>2</v>
+      </c>
+      <c r="B76" t="s">
+        <v>182</v>
+      </c>
+      <c r="D76" t="s">
+        <v>183</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A77">
+        <v>2</v>
+      </c>
+      <c r="B77" t="s">
+        <v>185</v>
+      </c>
+      <c r="D77" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A78">
+        <v>2</v>
+      </c>
+      <c r="B78" t="s">
+        <v>187</v>
+      </c>
+      <c r="D78" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A79">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>189</v>
+      </c>
+      <c r="D79" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A80">
+        <v>2</v>
+      </c>
+      <c r="B80" t="s">
+        <v>191</v>
+      </c>
+      <c r="C80" t="s">
+        <v>196</v>
+      </c>
+      <c r="D80" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A81">
+        <v>2</v>
+      </c>
+      <c r="B81" t="s">
+        <v>193</v>
+      </c>
+      <c r="C81" t="s">
+        <v>194</v>
+      </c>
+      <c r="D81" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A82">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>197</v>
+      </c>
+      <c r="D82" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A83">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>199</v>
+      </c>
+      <c r="C83" t="s">
+        <v>200</v>
+      </c>
+      <c r="D83" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A84">
+        <v>2</v>
+      </c>
+      <c r="B84" t="s">
+        <v>203</v>
+      </c>
+      <c r="D84" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A85">
+        <v>2</v>
+      </c>
+      <c r="B85" t="s">
+        <v>205</v>
+      </c>
+      <c r="D85" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A86">
+        <v>2</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="D86" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A87">
+        <v>2</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D87" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A88">
+        <v>2</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D88" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A89">
+        <v>2</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D89" t="s">
+        <v>214</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A90">
+        <v>2</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D90" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A91">
+        <v>2</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="D91" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A92">
+        <v>2</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D92" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A93">
+        <v>2</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D93" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A94">
+        <v>2</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="D94" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A95">
+        <v>2</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C95" t="s">
+        <v>228</v>
+      </c>
+      <c r="D95" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A96">
+        <v>2</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D96" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A97">
+        <v>2</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D97" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A98">
+        <v>2</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D98" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A99">
+        <v>2</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D99" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A100">
+        <v>2</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C100" t="s">
+        <v>238</v>
+      </c>
+      <c r="D100" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A101">
+        <v>2</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D101" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A102">
+        <v>2</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D102" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A103">
+        <v>2</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="D103" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A104">
+        <v>2</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D104" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A105">
+        <v>2</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="C105" t="s">
+        <v>249</v>
+      </c>
+      <c r="D105" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A106">
+        <v>2</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="D106" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A107">
+        <v>2</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D107" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A108">
+        <v>2</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D108" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A109">
+        <v>2</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D109" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A110">
+        <v>2</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="D110" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A111">
+        <v>2</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D111" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A112">
+        <v>2</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="D112" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A113">
+        <v>2</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D113" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A114">
+        <v>2</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="D114" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A115">
+        <v>2</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="D115" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A116">
+        <v>2</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="D116" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A117">
+        <v>2</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="D117" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A118">
+        <v>2</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D118" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A119">
+        <v>2</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C119" t="s">
+        <v>278</v>
+      </c>
+      <c r="D119" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A120">
+        <v>2</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="D120" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add clean Fre function
</commit_message>
<xml_diff>
--- a/READING/1_21_07.xlsx
+++ b/READING/1_21_07.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\READING\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDEE530F-49BC-4095-A58C-53EE5756E5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC642E25-4974-41AF-BA0A-DD88F8B22F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17520" yWindow="1005" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19215" yWindow="1005" windowWidth="19185" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="284">
   <si>
-    <t>Fre</t>
-  </si>
-  <si>
     <t>单词</t>
   </si>
   <si>
@@ -876,13 +873,17 @@
   </si>
   <si>
     <t>2</t>
+  </si>
+  <si>
+    <t>Fre</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -902,6 +903,13 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -939,9 +947,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1257,23 +1268,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.15">
@@ -1281,13 +1292,13 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.15">
@@ -1295,13 +1306,13 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.15">
@@ -1309,13 +1320,13 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
       <c r="F4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.15">
@@ -1323,16 +1334,16 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
       <c r="F5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.15">
@@ -1340,13 +1351,13 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
       <c r="F6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.15">
@@ -1354,16 +1365,16 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>20</v>
-      </c>
-      <c r="F7" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.15">
@@ -1371,13 +1382,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
         <v>22</v>
       </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.15">
@@ -1385,16 +1396,16 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
       <c r="F9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.15">
@@ -1402,13 +1413,13 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
         <v>26</v>
       </c>
-      <c r="D10" t="s">
-        <v>27</v>
-      </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.15">
@@ -1416,13 +1427,13 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
         <v>28</v>
       </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.15">
@@ -1430,16 +1441,16 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
         <v>30</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
       <c r="F12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.15">
@@ -1447,13 +1458,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
         <v>33</v>
       </c>
-      <c r="D13" t="s">
-        <v>34</v>
-      </c>
       <c r="F13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.15">
@@ -1461,16 +1472,16 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
         <v>35</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>36</v>
       </c>
-      <c r="D14" t="s">
-        <v>37</v>
-      </c>
       <c r="F14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.15">
@@ -1478,13 +1489,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
         <v>38</v>
       </c>
-      <c r="D15" t="s">
-        <v>39</v>
-      </c>
       <c r="F15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.15">
@@ -1492,13 +1503,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
         <v>40</v>
       </c>
-      <c r="D16" t="s">
-        <v>41</v>
-      </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.15">
@@ -1506,16 +1517,16 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
         <v>42</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="E17" t="s">
-        <v>44</v>
-      </c>
       <c r="F17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.15">
@@ -1523,13 +1534,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
         <v>45</v>
       </c>
-      <c r="D18" t="s">
-        <v>46</v>
-      </c>
       <c r="F18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.15">
@@ -1537,13 +1548,13 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
         <v>47</v>
       </c>
-      <c r="D19" t="s">
-        <v>48</v>
-      </c>
       <c r="F19" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.15">
@@ -1551,16 +1562,16 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
         <v>49</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>50</v>
       </c>
-      <c r="D20" t="s">
-        <v>51</v>
-      </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.15">
@@ -1568,13 +1579,13 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" t="s">
         <v>52</v>
       </c>
-      <c r="D21" t="s">
-        <v>53</v>
-      </c>
       <c r="F21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.15">
@@ -1582,13 +1593,13 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" t="s">
         <v>54</v>
       </c>
-      <c r="D22" t="s">
-        <v>55</v>
-      </c>
       <c r="F22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
@@ -1596,19 +1607,19 @@
         <v>4</v>
       </c>
       <c r="B23" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" t="s">
         <v>56</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>57</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>58</v>
       </c>
-      <c r="E23" t="s">
-        <v>59</v>
-      </c>
       <c r="F23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.15">
@@ -1616,16 +1627,16 @@
         <v>4</v>
       </c>
       <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" t="s">
         <v>60</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>61</v>
       </c>
-      <c r="D24" t="s">
-        <v>62</v>
-      </c>
       <c r="F24" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.15">
@@ -1633,16 +1644,16 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" t="s">
         <v>63</v>
       </c>
-      <c r="C25" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" t="s">
-        <v>64</v>
-      </c>
       <c r="F25" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.15">
@@ -1650,13 +1661,13 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" t="s">
         <v>65</v>
       </c>
-      <c r="D26" t="s">
-        <v>66</v>
-      </c>
       <c r="F26" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.15">
@@ -1664,13 +1675,13 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" t="s">
         <v>67</v>
       </c>
-      <c r="D27" t="s">
-        <v>68</v>
-      </c>
       <c r="F27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.15">
@@ -1678,16 +1689,16 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" t="s">
         <v>69</v>
       </c>
-      <c r="C28" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" t="s">
-        <v>70</v>
-      </c>
       <c r="F28" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.15">
@@ -1695,13 +1706,13 @@
         <v>4</v>
       </c>
       <c r="B29" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" t="s">
         <v>71</v>
       </c>
-      <c r="D29" t="s">
-        <v>72</v>
-      </c>
       <c r="F29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.15">
@@ -1709,16 +1720,16 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" t="s">
         <v>73</v>
       </c>
-      <c r="C30" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" t="s">
-        <v>74</v>
-      </c>
       <c r="F30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.15">
@@ -1726,13 +1737,13 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" t="s">
         <v>75</v>
       </c>
-      <c r="D31" t="s">
-        <v>76</v>
-      </c>
       <c r="F31" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.15">
@@ -1740,16 +1751,16 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" t="s">
         <v>77</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>78</v>
       </c>
-      <c r="D32" t="s">
-        <v>79</v>
-      </c>
       <c r="F32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.15">
@@ -1757,16 +1768,16 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" t="s">
         <v>80</v>
       </c>
-      <c r="C33" t="s">
-        <v>80</v>
-      </c>
-      <c r="D33" t="s">
-        <v>81</v>
-      </c>
       <c r="F33" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.15">
@@ -1774,13 +1785,13 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" t="s">
         <v>82</v>
       </c>
-      <c r="D34" t="s">
-        <v>83</v>
-      </c>
       <c r="F34" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.15">
@@ -1788,13 +1799,13 @@
         <v>3</v>
       </c>
       <c r="B35" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" t="s">
         <v>84</v>
       </c>
-      <c r="D35" t="s">
-        <v>85</v>
-      </c>
       <c r="F35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.15">
@@ -1802,16 +1813,16 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" t="s">
         <v>86</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>87</v>
       </c>
-      <c r="D36" t="s">
-        <v>88</v>
-      </c>
       <c r="F36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.15">
@@ -1819,13 +1830,13 @@
         <v>3</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F37" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.15">
@@ -1833,13 +1844,13 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38" t="s">
         <v>90</v>
       </c>
-      <c r="D38" t="s">
-        <v>91</v>
-      </c>
       <c r="F38" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.15">
@@ -1847,13 +1858,13 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" t="s">
         <v>92</v>
       </c>
-      <c r="D39" t="s">
-        <v>93</v>
-      </c>
       <c r="F39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.15">
@@ -1861,16 +1872,16 @@
         <v>3</v>
       </c>
       <c r="B40" t="s">
+        <v>93</v>
+      </c>
+      <c r="C40" t="s">
         <v>94</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>95</v>
       </c>
-      <c r="D40" t="s">
-        <v>96</v>
-      </c>
       <c r="F40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.15">
@@ -1878,13 +1889,13 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
+        <v>96</v>
+      </c>
+      <c r="D41" t="s">
         <v>97</v>
       </c>
-      <c r="D41" t="s">
-        <v>98</v>
-      </c>
       <c r="F41" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.15">
@@ -1892,13 +1903,13 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
+        <v>98</v>
+      </c>
+      <c r="D42" t="s">
         <v>99</v>
       </c>
-      <c r="D42" t="s">
-        <v>100</v>
-      </c>
       <c r="F42" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.15">
@@ -1906,13 +1917,13 @@
         <v>2</v>
       </c>
       <c r="B43" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" t="s">
         <v>101</v>
       </c>
-      <c r="D43" t="s">
-        <v>102</v>
-      </c>
       <c r="F43" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.15">
@@ -1920,16 +1931,16 @@
         <v>2</v>
       </c>
       <c r="B44" t="s">
+        <v>102</v>
+      </c>
+      <c r="C44" t="s">
         <v>103</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>104</v>
       </c>
-      <c r="D44" t="s">
-        <v>105</v>
-      </c>
       <c r="F44" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.15">
@@ -1937,16 +1948,16 @@
         <v>2</v>
       </c>
       <c r="B45" t="s">
+        <v>105</v>
+      </c>
+      <c r="C45" t="s">
         <v>106</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>107</v>
       </c>
-      <c r="D45" t="s">
-        <v>108</v>
-      </c>
       <c r="F45" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.15">
@@ -1954,16 +1965,16 @@
         <v>2</v>
       </c>
       <c r="B46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" t="s">
         <v>109</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>110</v>
       </c>
-      <c r="D46" t="s">
-        <v>111</v>
-      </c>
       <c r="F46" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.15">
@@ -1971,13 +1982,13 @@
         <v>2</v>
       </c>
       <c r="B47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" t="s">
         <v>112</v>
       </c>
-      <c r="D47" t="s">
-        <v>113</v>
-      </c>
       <c r="F47" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.15">
@@ -1985,13 +1996,13 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" t="s">
         <v>114</v>
       </c>
-      <c r="D48" t="s">
-        <v>115</v>
-      </c>
       <c r="F48" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.15">
@@ -1999,13 +2010,13 @@
         <v>2</v>
       </c>
       <c r="B49" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" t="s">
         <v>116</v>
       </c>
-      <c r="D49" t="s">
-        <v>117</v>
-      </c>
       <c r="F49" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.15">
@@ -2013,13 +2024,13 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50" t="s">
         <v>118</v>
       </c>
-      <c r="D50" t="s">
-        <v>119</v>
-      </c>
       <c r="F50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.15">
@@ -2027,13 +2038,13 @@
         <v>2</v>
       </c>
       <c r="B51" t="s">
+        <v>119</v>
+      </c>
+      <c r="D51" t="s">
         <v>120</v>
       </c>
-      <c r="D51" t="s">
-        <v>121</v>
-      </c>
       <c r="F51" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.15">
@@ -2041,13 +2052,13 @@
         <v>2</v>
       </c>
       <c r="B52" t="s">
+        <v>121</v>
+      </c>
+      <c r="D52" t="s">
         <v>122</v>
       </c>
-      <c r="D52" t="s">
-        <v>123</v>
-      </c>
       <c r="F52" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.15">
@@ -2055,13 +2066,13 @@
         <v>2</v>
       </c>
       <c r="B53" t="s">
+        <v>123</v>
+      </c>
+      <c r="D53" t="s">
         <v>124</v>
       </c>
-      <c r="D53" t="s">
-        <v>125</v>
-      </c>
       <c r="F53" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.15">
@@ -2069,13 +2080,13 @@
         <v>2</v>
       </c>
       <c r="B54" t="s">
+        <v>125</v>
+      </c>
+      <c r="D54" t="s">
         <v>126</v>
       </c>
-      <c r="D54" t="s">
-        <v>127</v>
-      </c>
       <c r="F54" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.15">
@@ -2083,13 +2094,13 @@
         <v>2</v>
       </c>
       <c r="B55" t="s">
+        <v>127</v>
+      </c>
+      <c r="D55" t="s">
         <v>128</v>
       </c>
-      <c r="D55" t="s">
-        <v>129</v>
-      </c>
       <c r="F55" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.15">
@@ -2097,13 +2108,13 @@
         <v>2</v>
       </c>
       <c r="B56" t="s">
+        <v>129</v>
+      </c>
+      <c r="D56" t="s">
         <v>130</v>
       </c>
-      <c r="D56" t="s">
-        <v>131</v>
-      </c>
       <c r="F56" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.15">
@@ -2111,13 +2122,13 @@
         <v>2</v>
       </c>
       <c r="B57" t="s">
+        <v>131</v>
+      </c>
+      <c r="D57" t="s">
         <v>132</v>
       </c>
-      <c r="D57" t="s">
-        <v>133</v>
-      </c>
       <c r="F57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.15">
@@ -2125,13 +2136,13 @@
         <v>2</v>
       </c>
       <c r="B58" t="s">
+        <v>133</v>
+      </c>
+      <c r="D58" t="s">
         <v>134</v>
       </c>
-      <c r="D58" t="s">
-        <v>135</v>
-      </c>
       <c r="F58" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.15">
@@ -2139,13 +2150,13 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
+        <v>135</v>
+      </c>
+      <c r="D59" t="s">
         <v>136</v>
       </c>
-      <c r="D59" t="s">
-        <v>137</v>
-      </c>
       <c r="F59" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
@@ -2153,13 +2164,13 @@
         <v>2</v>
       </c>
       <c r="B60" t="s">
+        <v>137</v>
+      </c>
+      <c r="D60" t="s">
         <v>138</v>
       </c>
-      <c r="D60" t="s">
-        <v>139</v>
-      </c>
       <c r="F60" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.15">
@@ -2167,13 +2178,13 @@
         <v>2</v>
       </c>
       <c r="B61" t="s">
+        <v>139</v>
+      </c>
+      <c r="D61" t="s">
         <v>140</v>
       </c>
-      <c r="D61" t="s">
-        <v>141</v>
-      </c>
       <c r="F61" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.15">
@@ -2181,13 +2192,13 @@
         <v>2</v>
       </c>
       <c r="B62" t="s">
+        <v>141</v>
+      </c>
+      <c r="D62" t="s">
         <v>142</v>
       </c>
-      <c r="D62" t="s">
-        <v>143</v>
-      </c>
       <c r="F62" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
@@ -2195,16 +2206,16 @@
         <v>2</v>
       </c>
       <c r="B63" t="s">
+        <v>143</v>
+      </c>
+      <c r="C63" t="s">
         <v>144</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>145</v>
       </c>
-      <c r="D63" t="s">
-        <v>146</v>
-      </c>
       <c r="F63" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.15">
@@ -2212,13 +2223,13 @@
         <v>2</v>
       </c>
       <c r="B64" t="s">
+        <v>146</v>
+      </c>
+      <c r="D64" t="s">
         <v>147</v>
       </c>
-      <c r="D64" t="s">
-        <v>148</v>
-      </c>
       <c r="F64" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.15">
@@ -2226,13 +2237,13 @@
         <v>2</v>
       </c>
       <c r="B65" t="s">
+        <v>148</v>
+      </c>
+      <c r="D65" t="s">
         <v>149</v>
       </c>
-      <c r="D65" t="s">
-        <v>150</v>
-      </c>
       <c r="F65" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.15">
@@ -2240,13 +2251,13 @@
         <v>3</v>
       </c>
       <c r="B66" t="s">
+        <v>150</v>
+      </c>
+      <c r="D66" t="s">
         <v>151</v>
       </c>
-      <c r="D66" t="s">
-        <v>152</v>
-      </c>
       <c r="F66" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.15">
@@ -2254,16 +2265,16 @@
         <v>2</v>
       </c>
       <c r="B67" t="s">
+        <v>152</v>
+      </c>
+      <c r="C67" t="s">
         <v>153</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>154</v>
       </c>
-      <c r="D67" t="s">
-        <v>155</v>
-      </c>
       <c r="F67" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.15">
@@ -2271,16 +2282,16 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
+        <v>155</v>
+      </c>
+      <c r="C68" t="s">
         <v>156</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>157</v>
       </c>
-      <c r="D68" t="s">
-        <v>158</v>
-      </c>
       <c r="F68" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.15">
@@ -2288,16 +2299,16 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
+        <v>158</v>
+      </c>
+      <c r="C69" t="s">
         <v>159</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>160</v>
       </c>
-      <c r="D69" t="s">
-        <v>161</v>
-      </c>
       <c r="F69" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.15">
@@ -2305,16 +2316,16 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" t="s">
         <v>162</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>163</v>
       </c>
-      <c r="D70" t="s">
-        <v>164</v>
-      </c>
       <c r="F70" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.15">
@@ -2322,13 +2333,13 @@
         <v>2</v>
       </c>
       <c r="B71" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D71" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F71" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.15">
@@ -2336,13 +2347,13 @@
         <v>2</v>
       </c>
       <c r="B72" t="s">
+        <v>165</v>
+      </c>
+      <c r="D72" t="s">
         <v>166</v>
       </c>
-      <c r="D72" t="s">
-        <v>167</v>
-      </c>
       <c r="F72" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.15">
@@ -2350,16 +2361,16 @@
         <v>2</v>
       </c>
       <c r="B73" t="s">
+        <v>167</v>
+      </c>
+      <c r="C73" t="s">
         <v>168</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>169</v>
       </c>
-      <c r="D73" t="s">
-        <v>170</v>
-      </c>
       <c r="F73" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.15">
@@ -2367,16 +2378,16 @@
         <v>2</v>
       </c>
       <c r="B74" t="s">
+        <v>170</v>
+      </c>
+      <c r="D74" t="s">
         <v>171</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>172</v>
       </c>
-      <c r="E74" t="s">
-        <v>173</v>
-      </c>
       <c r="F74" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.15">
@@ -2384,13 +2395,13 @@
         <v>3</v>
       </c>
       <c r="B75" t="s">
+        <v>173</v>
+      </c>
+      <c r="D75" t="s">
         <v>174</v>
       </c>
-      <c r="D75" t="s">
-        <v>175</v>
-      </c>
       <c r="F75" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.15">
@@ -2398,16 +2409,16 @@
         <v>2</v>
       </c>
       <c r="B76" t="s">
+        <v>175</v>
+      </c>
+      <c r="C76" t="s">
         <v>176</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>177</v>
       </c>
-      <c r="D76" t="s">
-        <v>178</v>
-      </c>
       <c r="F76" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.15">
@@ -2415,13 +2426,13 @@
         <v>2</v>
       </c>
       <c r="B77" t="s">
+        <v>178</v>
+      </c>
+      <c r="D77" t="s">
         <v>179</v>
       </c>
-      <c r="D77" t="s">
-        <v>180</v>
-      </c>
       <c r="F77" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.15">
@@ -2429,13 +2440,13 @@
         <v>2</v>
       </c>
       <c r="B78" t="s">
+        <v>180</v>
+      </c>
+      <c r="D78" t="s">
         <v>181</v>
       </c>
-      <c r="D78" t="s">
-        <v>182</v>
-      </c>
       <c r="F78" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.15">
@@ -2443,13 +2454,13 @@
         <v>2</v>
       </c>
       <c r="B79" t="s">
+        <v>182</v>
+      </c>
+      <c r="D79" t="s">
         <v>183</v>
       </c>
-      <c r="D79" t="s">
-        <v>184</v>
-      </c>
       <c r="F79" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.15">
@@ -2457,13 +2468,13 @@
         <v>2</v>
       </c>
       <c r="B80" t="s">
+        <v>184</v>
+      </c>
+      <c r="D80" t="s">
         <v>185</v>
       </c>
-      <c r="D80" t="s">
-        <v>186</v>
-      </c>
       <c r="F80" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.15">
@@ -2471,13 +2482,13 @@
         <v>2</v>
       </c>
       <c r="B81" t="s">
+        <v>186</v>
+      </c>
+      <c r="D81" t="s">
         <v>187</v>
       </c>
-      <c r="D81" t="s">
-        <v>188</v>
-      </c>
       <c r="F81" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.15">
@@ -2485,13 +2496,13 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
+        <v>188</v>
+      </c>
+      <c r="D82" t="s">
         <v>189</v>
       </c>
-      <c r="D82" t="s">
-        <v>190</v>
-      </c>
       <c r="F82" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.15">
@@ -2499,13 +2510,13 @@
         <v>2</v>
       </c>
       <c r="B83" t="s">
+        <v>190</v>
+      </c>
+      <c r="D83" t="s">
         <v>191</v>
       </c>
-      <c r="D83" t="s">
-        <v>192</v>
-      </c>
       <c r="F83" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.15">
@@ -2513,13 +2524,13 @@
         <v>2</v>
       </c>
       <c r="B84" t="s">
+        <v>192</v>
+      </c>
+      <c r="D84" t="s">
         <v>193</v>
       </c>
-      <c r="D84" t="s">
-        <v>194</v>
-      </c>
       <c r="F84" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.15">
@@ -2527,13 +2538,13 @@
         <v>2</v>
       </c>
       <c r="B85" t="s">
+        <v>194</v>
+      </c>
+      <c r="D85" t="s">
         <v>195</v>
       </c>
-      <c r="D85" t="s">
-        <v>196</v>
-      </c>
       <c r="F85" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.15">
@@ -2541,16 +2552,16 @@
         <v>1</v>
       </c>
       <c r="B86" t="s">
+        <v>196</v>
+      </c>
+      <c r="C86" t="s">
+        <v>196</v>
+      </c>
+      <c r="D86" t="s">
         <v>197</v>
       </c>
-      <c r="C86" t="s">
-        <v>197</v>
-      </c>
-      <c r="D86" t="s">
-        <v>198</v>
-      </c>
       <c r="F86" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.15">
@@ -2558,16 +2569,16 @@
         <v>1</v>
       </c>
       <c r="B87" t="s">
+        <v>198</v>
+      </c>
+      <c r="C87" t="s">
         <v>199</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>200</v>
       </c>
-      <c r="D87" t="s">
-        <v>201</v>
-      </c>
       <c r="F87" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.15">
@@ -2575,16 +2586,16 @@
         <v>1</v>
       </c>
       <c r="B88" t="s">
+        <v>201</v>
+      </c>
+      <c r="C88" t="s">
         <v>202</v>
       </c>
-      <c r="C88" t="s">
-        <v>203</v>
-      </c>
       <c r="D88" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F88" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.15">
@@ -2592,16 +2603,16 @@
         <v>1</v>
       </c>
       <c r="B89" t="s">
+        <v>203</v>
+      </c>
+      <c r="C89" t="s">
+        <v>203</v>
+      </c>
+      <c r="D89" t="s">
         <v>204</v>
       </c>
-      <c r="C89" t="s">
-        <v>204</v>
-      </c>
-      <c r="D89" t="s">
-        <v>205</v>
-      </c>
       <c r="F89" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.15">
@@ -2609,16 +2620,16 @@
         <v>1</v>
       </c>
       <c r="B90" t="s">
+        <v>205</v>
+      </c>
+      <c r="D90" t="s">
         <v>206</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>207</v>
       </c>
-      <c r="E90" t="s">
-        <v>208</v>
-      </c>
       <c r="F90" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.15">
@@ -2626,16 +2637,16 @@
         <v>1</v>
       </c>
       <c r="B91" t="s">
+        <v>208</v>
+      </c>
+      <c r="C91" t="s">
         <v>209</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
         <v>210</v>
       </c>
-      <c r="D91" t="s">
-        <v>211</v>
-      </c>
       <c r="F91" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.15">
@@ -2643,16 +2654,16 @@
         <v>1</v>
       </c>
       <c r="B92" t="s">
+        <v>211</v>
+      </c>
+      <c r="C92" t="s">
         <v>212</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
         <v>213</v>
       </c>
-      <c r="D92" t="s">
-        <v>214</v>
-      </c>
       <c r="F92" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.15">
@@ -2660,16 +2671,16 @@
         <v>1</v>
       </c>
       <c r="B93" t="s">
+        <v>214</v>
+      </c>
+      <c r="C93" t="s">
+        <v>214</v>
+      </c>
+      <c r="D93" t="s">
         <v>215</v>
       </c>
-      <c r="C93" t="s">
-        <v>215</v>
-      </c>
-      <c r="D93" t="s">
-        <v>216</v>
-      </c>
       <c r="F93" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.15">
@@ -2677,16 +2688,16 @@
         <v>0</v>
       </c>
       <c r="B94" t="s">
+        <v>216</v>
+      </c>
+      <c r="C94" t="s">
+        <v>216</v>
+      </c>
+      <c r="D94" t="s">
         <v>217</v>
       </c>
-      <c r="C94" t="s">
-        <v>217</v>
-      </c>
-      <c r="D94" t="s">
-        <v>218</v>
-      </c>
       <c r="F94" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.15">
@@ -2694,16 +2705,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
+        <v>218</v>
+      </c>
+      <c r="C95" t="s">
         <v>219</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
         <v>220</v>
       </c>
-      <c r="D95" t="s">
-        <v>221</v>
-      </c>
       <c r="F95" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.15">
@@ -2711,16 +2722,16 @@
         <v>0</v>
       </c>
       <c r="B96" t="s">
+        <v>221</v>
+      </c>
+      <c r="C96" t="s">
+        <v>221</v>
+      </c>
+      <c r="D96" t="s">
         <v>222</v>
       </c>
-      <c r="C96" t="s">
-        <v>222</v>
-      </c>
-      <c r="D96" t="s">
-        <v>223</v>
-      </c>
       <c r="F96" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.15">
@@ -2728,16 +2739,16 @@
         <v>0</v>
       </c>
       <c r="B97" t="s">
+        <v>223</v>
+      </c>
+      <c r="C97" t="s">
+        <v>223</v>
+      </c>
+      <c r="D97" t="s">
         <v>224</v>
       </c>
-      <c r="C97" t="s">
-        <v>224</v>
-      </c>
-      <c r="D97" t="s">
-        <v>225</v>
-      </c>
       <c r="F97" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.15">
@@ -2745,16 +2756,16 @@
         <v>0</v>
       </c>
       <c r="B98" t="s">
+        <v>225</v>
+      </c>
+      <c r="C98" t="s">
+        <v>225</v>
+      </c>
+      <c r="D98" t="s">
         <v>226</v>
       </c>
-      <c r="C98" t="s">
-        <v>226</v>
-      </c>
-      <c r="D98" t="s">
-        <v>227</v>
-      </c>
       <c r="F98" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.15">
@@ -2762,16 +2773,16 @@
         <v>0</v>
       </c>
       <c r="B99" t="s">
+        <v>227</v>
+      </c>
+      <c r="C99" t="s">
+        <v>227</v>
+      </c>
+      <c r="D99" t="s">
         <v>228</v>
       </c>
-      <c r="C99" t="s">
-        <v>228</v>
-      </c>
-      <c r="D99" t="s">
-        <v>229</v>
-      </c>
       <c r="F99" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.15">
@@ -2779,16 +2790,16 @@
         <v>0</v>
       </c>
       <c r="B100" t="s">
+        <v>229</v>
+      </c>
+      <c r="C100" t="s">
         <v>230</v>
       </c>
-      <c r="C100" t="s">
+      <c r="D100" t="s">
         <v>231</v>
       </c>
-      <c r="D100" t="s">
-        <v>232</v>
-      </c>
       <c r="F100" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.15">
@@ -2796,19 +2807,19 @@
         <v>0</v>
       </c>
       <c r="B101" t="s">
+        <v>232</v>
+      </c>
+      <c r="C101" t="s">
+        <v>232</v>
+      </c>
+      <c r="D101" t="s">
         <v>233</v>
       </c>
-      <c r="C101" t="s">
-        <v>233</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="E101" t="s">
         <v>234</v>
       </c>
-      <c r="E101" t="s">
-        <v>235</v>
-      </c>
       <c r="F101" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.15">
@@ -2816,16 +2827,16 @@
         <v>0</v>
       </c>
       <c r="B102" t="s">
+        <v>235</v>
+      </c>
+      <c r="C102" t="s">
+        <v>235</v>
+      </c>
+      <c r="D102" t="s">
         <v>236</v>
       </c>
-      <c r="C102" t="s">
-        <v>236</v>
-      </c>
-      <c r="D102" t="s">
-        <v>237</v>
-      </c>
       <c r="F102" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.15">
@@ -2833,16 +2844,16 @@
         <v>0</v>
       </c>
       <c r="B103" t="s">
+        <v>237</v>
+      </c>
+      <c r="C103" t="s">
         <v>238</v>
       </c>
-      <c r="C103" t="s">
+      <c r="D103" t="s">
         <v>239</v>
       </c>
-      <c r="D103" t="s">
-        <v>240</v>
-      </c>
       <c r="F103" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.15">
@@ -2850,16 +2861,16 @@
         <v>0</v>
       </c>
       <c r="B104" t="s">
+        <v>240</v>
+      </c>
+      <c r="C104" t="s">
+        <v>225</v>
+      </c>
+      <c r="D104" t="s">
         <v>241</v>
       </c>
-      <c r="C104" t="s">
-        <v>226</v>
-      </c>
-      <c r="D104" t="s">
-        <v>242</v>
-      </c>
       <c r="F104" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.15">
@@ -2867,16 +2878,16 @@
         <v>0</v>
       </c>
       <c r="B105" t="s">
+        <v>242</v>
+      </c>
+      <c r="C105" t="s">
+        <v>242</v>
+      </c>
+      <c r="D105" t="s">
         <v>243</v>
       </c>
-      <c r="C105" t="s">
-        <v>243</v>
-      </c>
-      <c r="D105" t="s">
-        <v>244</v>
-      </c>
       <c r="F105" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.15">
@@ -2884,16 +2895,16 @@
         <v>0</v>
       </c>
       <c r="B106" t="s">
+        <v>244</v>
+      </c>
+      <c r="C106" t="s">
         <v>245</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>246</v>
       </c>
-      <c r="D106" t="s">
-        <v>247</v>
-      </c>
       <c r="F106" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.15">
@@ -2901,13 +2912,13 @@
         <v>0</v>
       </c>
       <c r="B107" t="s">
+        <v>247</v>
+      </c>
+      <c r="D107" t="s">
         <v>248</v>
       </c>
-      <c r="D107" t="s">
-        <v>249</v>
-      </c>
       <c r="F107" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.15">
@@ -2915,16 +2926,16 @@
         <v>0</v>
       </c>
       <c r="B108" t="s">
+        <v>249</v>
+      </c>
+      <c r="D108" t="s">
         <v>250</v>
       </c>
-      <c r="D108" t="s">
+      <c r="E108" t="s">
         <v>251</v>
       </c>
-      <c r="E108" t="s">
-        <v>252</v>
-      </c>
       <c r="F108" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.15">
@@ -2932,16 +2943,16 @@
         <v>0</v>
       </c>
       <c r="B109" t="s">
+        <v>252</v>
+      </c>
+      <c r="C109" t="s">
         <v>253</v>
       </c>
-      <c r="C109" t="s">
+      <c r="D109" t="s">
         <v>254</v>
       </c>
-      <c r="D109" t="s">
-        <v>255</v>
-      </c>
       <c r="F109" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.15">
@@ -2949,13 +2960,13 @@
         <v>0</v>
       </c>
       <c r="B110" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D110" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F110" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.15">
@@ -2963,16 +2974,16 @@
         <v>0</v>
       </c>
       <c r="B111" t="s">
+        <v>256</v>
+      </c>
+      <c r="C111" t="s">
         <v>257</v>
       </c>
-      <c r="C111" t="s">
+      <c r="D111" t="s">
         <v>258</v>
       </c>
-      <c r="D111" t="s">
-        <v>259</v>
-      </c>
       <c r="F111" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.15">
@@ -2980,13 +2991,13 @@
         <v>0</v>
       </c>
       <c r="B112" t="s">
+        <v>259</v>
+      </c>
+      <c r="D112" t="s">
         <v>260</v>
       </c>
-      <c r="D112" t="s">
-        <v>261</v>
-      </c>
       <c r="F112" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.15">
@@ -2994,16 +3005,16 @@
         <v>0</v>
       </c>
       <c r="B113" t="s">
+        <v>261</v>
+      </c>
+      <c r="C113" t="s">
+        <v>261</v>
+      </c>
+      <c r="D113" t="s">
         <v>262</v>
       </c>
-      <c r="C113" t="s">
-        <v>262</v>
-      </c>
-      <c r="D113" t="s">
-        <v>263</v>
-      </c>
       <c r="F113" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.15">
@@ -3011,16 +3022,16 @@
         <v>0</v>
       </c>
       <c r="B114" t="s">
+        <v>263</v>
+      </c>
+      <c r="D114" t="s">
         <v>264</v>
       </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
         <v>265</v>
       </c>
-      <c r="E114" t="s">
-        <v>266</v>
-      </c>
       <c r="F114" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.15">
@@ -3028,16 +3039,16 @@
         <v>0</v>
       </c>
       <c r="B115" t="s">
+        <v>266</v>
+      </c>
+      <c r="C115" t="s">
+        <v>266</v>
+      </c>
+      <c r="D115" t="s">
         <v>267</v>
       </c>
-      <c r="C115" t="s">
-        <v>267</v>
-      </c>
-      <c r="D115" t="s">
-        <v>268</v>
-      </c>
       <c r="F115" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.15">
@@ -3045,16 +3056,16 @@
         <v>0</v>
       </c>
       <c r="B116" t="s">
+        <v>268</v>
+      </c>
+      <c r="C116" t="s">
+        <v>268</v>
+      </c>
+      <c r="D116" t="s">
         <v>269</v>
       </c>
-      <c r="C116" t="s">
-        <v>269</v>
-      </c>
-      <c r="D116" t="s">
-        <v>270</v>
-      </c>
       <c r="F116" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.15">
@@ -3062,16 +3073,16 @@
         <v>0</v>
       </c>
       <c r="B117" t="s">
+        <v>270</v>
+      </c>
+      <c r="C117" t="s">
         <v>271</v>
       </c>
-      <c r="C117" t="s">
+      <c r="D117" t="s">
         <v>272</v>
       </c>
-      <c r="D117" t="s">
-        <v>273</v>
-      </c>
       <c r="F117" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.15">
@@ -3079,16 +3090,16 @@
         <v>0</v>
       </c>
       <c r="B118" t="s">
+        <v>273</v>
+      </c>
+      <c r="C118" t="s">
         <v>274</v>
       </c>
-      <c r="C118" t="s">
+      <c r="D118" t="s">
         <v>275</v>
       </c>
-      <c r="D118" t="s">
-        <v>276</v>
-      </c>
       <c r="F118" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.15">
@@ -3096,13 +3107,13 @@
         <v>1</v>
       </c>
       <c r="B119" t="s">
+        <v>276</v>
+      </c>
+      <c r="D119" t="s">
         <v>277</v>
       </c>
-      <c r="D119" t="s">
-        <v>278</v>
-      </c>
       <c r="F119" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.15">
@@ -3110,16 +3121,16 @@
         <v>0</v>
       </c>
       <c r="B120" t="s">
+        <v>278</v>
+      </c>
+      <c r="C120" t="s">
+        <v>278</v>
+      </c>
+      <c r="D120" t="s">
         <v>279</v>
       </c>
-      <c r="C120" t="s">
-        <v>279</v>
-      </c>
-      <c r="D120" t="s">
-        <v>280</v>
-      </c>
       <c r="F120" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.15">
@@ -3127,13 +3138,13 @@
         <v>1</v>
       </c>
       <c r="B121" t="s">
+        <v>280</v>
+      </c>
+      <c r="D121" t="s">
         <v>281</v>
       </c>
-      <c r="D121" t="s">
+      <c r="F121" t="s">
         <v>282</v>
-      </c>
-      <c r="F121" t="s">
-        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>